<commit_message>
use quality instead of test - tests work in iRODS!
</commit_message>
<xml_diff>
--- a/tests/testdata/testdata.xlsx
+++ b/tests/testdata/testdata.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27531"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu-22.04\home\jef\repositories\gitea\foz\mango-metadata-from-tables\testdata\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-24.04\home\mariana\repos\gitea\foz\mango-metadata-from-tables\tests\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{DD6A3C82-373F-4A40-8BAD-C22E77AC7B0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C351429F-170D-4CF0-8086-82D9C65C18C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14016" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="15" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -39,15 +39,6 @@
     <t>shape</t>
   </si>
   <si>
-    <t>/icts/home/datateam_icts_icts_test/mango-metadata-from-tables/file1.txt</t>
-  </si>
-  <si>
-    <t>/icts/home/datateam_icts_icts_test/mango-metadata-from-tables/file2.txt</t>
-  </si>
-  <si>
-    <t>/icts/home/datateam_icts_icts_test/mango-metadata-from-tables/file3.txt</t>
-  </si>
-  <si>
     <t>small</t>
   </si>
   <si>
@@ -73,6 +64,15 @@
   </si>
   <si>
     <t>square</t>
+  </si>
+  <si>
+    <t>/icts/home/datateam_icts_icts_quality/mango-metadata-from-tables/file1.txt</t>
+  </si>
+  <si>
+    <t>/icts/home/datateam_icts_icts_quality/mango-metadata-from-tables/file2.txt</t>
+  </si>
+  <si>
+    <t>/icts/home/datateam_icts_icts_quality/mango-metadata-from-tables/file3.txt</t>
   </si>
 </sst>
 </file>
@@ -391,12 +391,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="61.33203125" customWidth="1"/>
+    <col min="1" max="1" width="61.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -410,46 +410,46 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B2" t="s">
         <v>4</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>7</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>10</v>
       </c>
-      <c r="D2" t="s">
-        <v>13</v>
-      </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B3" t="s">
         <v>5</v>
       </c>
-      <c r="B3" t="s">
+      <c r="C3" t="s">
         <v>8</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
         <v>11</v>
       </c>
-      <c r="D3" t="s">
-        <v>14</v>
-      </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B4" t="s">
         <v>6</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" t="s">
         <v>9</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>12</v>
-      </c>
-      <c r="D4" t="s">
-        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
First merge from development (#5)
* update dependencies
- upgrade to latest mango-mdschema version
- fix pytest version for compatibility with pytest-cases

* Split function to apply metadata from click command
* use schemas with realm and name, see #42

* write tests for schemas in iRODS
* add ci/cd

---------

Co-authored-by: Jef Scheepers <jef.scheepers@kuleuven.be>
</commit_message>
<xml_diff>
--- a/tests/testdata/testdata.xlsx
+++ b/tests/testdata/testdata.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27531"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu-22.04\home\jef\repositories\gitea\foz\mango-metadata-from-tables\testdata\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-24.04\home\mariana\repos\gitea\foz\mango-metadata-from-tables\tests\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{DD6A3C82-373F-4A40-8BAD-C22E77AC7B0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C351429F-170D-4CF0-8086-82D9C65C18C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14016" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="15" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -39,15 +39,6 @@
     <t>shape</t>
   </si>
   <si>
-    <t>/icts/home/datateam_icts_icts_test/mango-metadata-from-tables/file1.txt</t>
-  </si>
-  <si>
-    <t>/icts/home/datateam_icts_icts_test/mango-metadata-from-tables/file2.txt</t>
-  </si>
-  <si>
-    <t>/icts/home/datateam_icts_icts_test/mango-metadata-from-tables/file3.txt</t>
-  </si>
-  <si>
     <t>small</t>
   </si>
   <si>
@@ -73,6 +64,15 @@
   </si>
   <si>
     <t>square</t>
+  </si>
+  <si>
+    <t>/icts/home/datateam_icts_icts_quality/mango-metadata-from-tables/file1.txt</t>
+  </si>
+  <si>
+    <t>/icts/home/datateam_icts_icts_quality/mango-metadata-from-tables/file2.txt</t>
+  </si>
+  <si>
+    <t>/icts/home/datateam_icts_icts_quality/mango-metadata-from-tables/file3.txt</t>
   </si>
 </sst>
 </file>
@@ -391,12 +391,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="61.33203125" customWidth="1"/>
+    <col min="1" max="1" width="61.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -410,46 +410,46 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B2" t="s">
         <v>4</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>7</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>10</v>
       </c>
-      <c r="D2" t="s">
-        <v>13</v>
-      </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B3" t="s">
         <v>5</v>
       </c>
-      <c r="B3" t="s">
+      <c r="C3" t="s">
         <v>8</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
         <v>11</v>
       </c>
-      <c r="D3" t="s">
-        <v>14</v>
-      </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B4" t="s">
         <v>6</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" t="s">
         <v>9</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>12</v>
-      </c>
-      <c r="D4" t="s">
-        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>